<commit_message>
Sincronización con el repositorio main 6 de Marzo 2026
</commit_message>
<xml_diff>
--- a/indicadores/ARG-CAME_out.xlsx
+++ b/indicadores/ARG-CAME_out.xlsx
@@ -106,13 +106,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">21/01/2026</t>
+    <t xml:space="preserve">04/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">ysonder</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1450,7 +1450,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.554440242510697</v>
+        <v>0.54502488435189</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1508,7 +1508,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.30740398251532</v>
+        <v>0.297052124562791</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1578,7 +1578,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0519050075614253</v>
+        <v>0.0775073273367491</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1608,7 +1608,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.00362753363518894</v>
+        <v>0.00178031181122585</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -13275,7 +13275,7 @@
         <v>282</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0686868887254674</v>
+        <v>-0.0781346713203792</v>
       </c>
     </row>
     <row r="6">
@@ -13283,7 +13283,7 @@
         <v>283</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0684026671030166</v>
+        <v>-0.0781963399869195</v>
       </c>
     </row>
     <row r="7">
@@ -13291,7 +13291,7 @@
         <v>284</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.0797996272607916</v>
+        <v>-0.0844821227032373</v>
       </c>
     </row>
     <row r="8">
@@ -13299,7 +13299,7 @@
         <v>285</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>-0.108000633519204</v>
+        <v>-0.108744671240276</v>
       </c>
     </row>
     <row r="9">
@@ -13307,7 +13307,7 @@
         <v>286</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>-0.0713118534019263</v>
+        <v>-0.0702800479497654</v>
       </c>
     </row>
     <row r="10">
@@ -13315,7 +13315,7 @@
         <v>287</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.0716221717557546</v>
+        <v>0.073075264665278</v>
       </c>
     </row>
     <row r="11">
@@ -13323,7 +13323,7 @@
         <v>288</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.254296341521941</v>
+        <v>0.254099436353175</v>
       </c>
     </row>
     <row r="12">
@@ -13331,7 +13331,7 @@
         <v>289</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.411942144332672</v>
+        <v>0.408528412751203</v>
       </c>
     </row>
     <row r="13">
@@ -13339,7 +13339,7 @@
         <v>290</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.514187574849594</v>
+        <v>0.506244856335707</v>
       </c>
     </row>
     <row r="14">
@@ -13347,7 +13347,7 @@
         <v>291</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.554440242510697</v>
+        <v>0.54502488435189</v>
       </c>
     </row>
     <row r="15">
@@ -13355,7 +13355,7 @@
         <v>292</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.490564565335413</v>
+        <v>0.4887821646558</v>
       </c>
     </row>
     <row r="16">
@@ -13363,7 +13363,7 @@
         <v>293</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.344638722092969</v>
+        <v>0.347403018851958</v>
       </c>
     </row>
     <row r="17">
@@ -13371,7 +13371,7 @@
         <v>294</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.253132337963935</v>
+        <v>0.252732079350329</v>
       </c>
     </row>
     <row r="18">
@@ -13379,7 +13379,7 @@
         <v>295</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.225373036814731</v>
+        <v>0.22291401101774</v>
       </c>
     </row>
     <row r="19">
@@ -13387,7 +13387,7 @@
         <v>296</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.15184476018145</v>
+        <v>0.153567609371855</v>
       </c>
     </row>
     <row r="20">
@@ -13395,7 +13395,7 @@
         <v>297</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0523816113196551</v>
+        <v>0.0597851585306625</v>
       </c>
     </row>
     <row r="21">
@@ -13403,7 +13403,7 @@
         <v>298</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0510720144408793</v>
+        <v>-0.0469622008738864</v>
       </c>
     </row>
     <row r="22">
@@ -13411,7 +13411,7 @@
         <v>299</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.186525213469563</v>
+        <v>-0.184956547899453</v>
       </c>
     </row>
     <row r="23">
@@ -13419,7 +13419,7 @@
         <v>300</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.298643826523538</v>
+        <v>-0.297077513870126</v>
       </c>
     </row>
     <row r="24">
@@ -13447,237 +13447,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2876B2DA-494D-4B1A-8E67-5D5B145D7957}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63046971-5FB7-41A0-A881-DE6B1697A3A6}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5C5135E-DB29-494A-9B72-975D454D52CF}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | ARG-CAME | 2026-06-17 08:36:25.909834
</commit_message>
<xml_diff>
--- a/indicadores/ARG-CAME_out.xlsx
+++ b/indicadores/ARG-CAME_out.xlsx
@@ -107,7 +107,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">16/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -13791,237 +13791,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10CE3BED-7CF9-4514-BAEC-1924030B2E25}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025729D7-759A-4AA7-9337-1A0E4C0FB780}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64CAFEA2-4727-4FBD-95C7-11A62291C696}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | ARG-CAME | 2026-06-17 12:10:25.037918
</commit_message>
<xml_diff>
--- a/indicadores/ARG-CAME_out.xlsx
+++ b/indicadores/ARG-CAME_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="322">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Argentina</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -113,7 +119,7 @@
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1476,9 +1482,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1489,7 +1499,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1503,7 +1513,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -1519,7 +1529,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1547,7 +1557,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1561,7 +1571,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -1589,7 +1599,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1603,7 +1613,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1617,7 +1627,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1631,7 +1641,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -1647,7 +1657,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1661,7 +1671,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -1809,10 +1819,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1825,10 +1835,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1852,66 +1862,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>99.4134897360704</v>
@@ -1964,7 +1974,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>94.6236559139785</v>
@@ -2021,7 +2031,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>94.4281524926686</v>
@@ -2078,7 +2088,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>91.4956011730205</v>
@@ -2135,7 +2145,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>90.811339198436</v>
@@ -2192,7 +2202,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>95.9921798631476</v>
@@ -2249,7 +2259,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>100</v>
@@ -2306,7 +2316,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>101.066098081023</v>
@@ -2363,7 +2373,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>101.705756929638</v>
@@ -2420,7 +2430,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>104.157782515991</v>
@@ -2477,7 +2487,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>103.304904051173</v>
@@ -2534,7 +2544,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>111.194029850746</v>
@@ -2591,7 +2601,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>108.422174840085</v>
@@ -2650,7 +2660,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>103.19829424307</v>
@@ -2709,7 +2719,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>102.985074626866</v>
@@ -2768,7 +2778,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>99.7867803837953</v>
@@ -2827,7 +2837,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>99.0405117270789</v>
@@ -2886,7 +2896,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>104.690831556503</v>
@@ -2945,7 +2955,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>109.061833688699</v>
@@ -3004,7 +3014,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>104.477611940299</v>
@@ -3063,7 +3073,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>105.01066098081</v>
@@ -3122,7 +3132,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>109.488272921109</v>
@@ -3181,7 +3191,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>104.157782515991</v>
@@ -3240,7 +3250,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>108.315565031983</v>
@@ -3299,7 +3309,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>102.558635394456</v>
@@ -3358,7 +3368,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>99.680170575693</v>
@@ -3417,7 +3427,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>98.9339019189765</v>
@@ -3476,7 +3486,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>98.6140724946695</v>
@@ -3535,7 +3545,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>97.7611940298508</v>
@@ -3594,7 +3604,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>97.228144989339</v>
@@ -3653,7 +3663,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>96.3752665245203</v>
@@ -3712,7 +3722,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>96.6950959488273</v>
@@ -3771,7 +3781,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>97.8678038379531</v>
@@ -3830,7 +3840,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>100.959488272921</v>
@@ -3889,7 +3899,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>101.38592750533</v>
@@ -3948,7 +3958,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>108.742004264392</v>
@@ -4007,7 +4017,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>108.208955223881</v>
@@ -4066,7 +4076,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>109.594882729211</v>
@@ -4125,7 +4135,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>108.955223880597</v>
@@ -4184,7 +4194,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>108.315565031983</v>
@@ -4243,7 +4253,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>108.422174840085</v>
@@ -4302,7 +4312,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>108.528784648188</v>
@@ -4361,7 +4371,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>108.422174840085</v>
@@ -4420,7 +4430,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>109.168443496802</v>
@@ -4479,7 +4489,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>109.168443496802</v>
@@ -4538,7 +4548,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>109.488272921109</v>
@@ -4597,7 +4607,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>108.422174840085</v>
@@ -4656,7 +4666,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>109.914712153518</v>
@@ -4715,7 +4725,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>104.157782515991</v>
@@ -4774,7 +4784,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>101.81236673774</v>
@@ -4833,7 +4843,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>100.426439232409</v>
@@ -4892,7 +4902,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>99.5735607675906</v>
@@ -4951,7 +4961,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>96.8017057569296</v>
@@ -5010,7 +5020,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>96.1620469083156</v>
@@ -5069,7 +5079,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>97.9744136460555</v>
@@ -5128,7 +5138,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>98.7206823027719</v>
@@ -5187,7 +5197,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>98.4008528784648</v>
@@ -5246,7 +5256,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>97.8678038379531</v>
@@ -5305,7 +5315,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>97.5479744136461</v>
@@ -5364,7 +5374,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>100.852878464819</v>
@@ -5423,7 +5433,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>103.944562899787</v>
@@ -5482,7 +5492,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>102.238805970149</v>
@@ -5541,7 +5551,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>101.918976545842</v>
@@ -5600,7 +5610,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>102.558635394456</v>
@@ -5659,7 +5669,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>104.157782515991</v>
@@ -5718,7 +5728,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>105.117270788913</v>
@@ -5777,7 +5787,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>104.904051172708</v>
@@ -5836,7 +5846,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>106.289978678038</v>
@@ -5895,7 +5905,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>106.503198294243</v>
@@ -5954,7 +5964,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>108.315565031983</v>
@@ -6013,7 +6023,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>107.036247334755</v>
@@ -6072,7 +6082,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>107.782515991471</v>
@@ -6131,7 +6141,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>105.543710021322</v>
@@ -6190,7 +6200,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>105.01066098081</v>
@@ -6249,7 +6259,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>104.477611940299</v>
@@ -6308,7 +6318,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>103.411513859275</v>
@@ -6367,7 +6377,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>101.492537313433</v>
@@ -6426,7 +6436,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>102.132196162047</v>
@@ -6485,7 +6495,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>100.426439232409</v>
@@ -6544,7 +6554,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>98.0810234541578</v>
@@ -6603,7 +6613,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>97.8678038379531</v>
@@ -6662,7 +6672,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>96.588486140725</v>
@@ -6721,7 +6731,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>89.9786780383795</v>
@@ -6780,7 +6790,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>96.0554371002132</v>
@@ -6839,7 +6849,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>95.9488272921109</v>
@@ -6898,7 +6908,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>93.9232409381663</v>
@@ -6957,7 +6967,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>94.5628997867804</v>
@@ -7016,7 +7026,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>92.3240938166311</v>
@@ -7075,7 +7085,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>91.5778251599147</v>
@@ -7134,7 +7144,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>93.6034115138593</v>
@@ -7193,7 +7203,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>98.6140724946695</v>
@@ -7252,7 +7262,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>86.7803837953092</v>
@@ -7311,7 +7321,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>91.1513859275053</v>
@@ -7370,7 +7380,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>94.2430703624734</v>
@@ -7429,7 +7439,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>99.0405117270789</v>
@@ -7488,7 +7498,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>102.558635394456</v>
@@ -7547,7 +7557,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>102.878464818763</v>
@@ -7606,7 +7616,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>105.43710021322</v>
@@ -7665,7 +7675,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>54.6908315565032</v>
@@ -7724,7 +7734,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>45.2025586353944</v>
@@ -7783,7 +7793,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>52.4520255863539</v>
@@ -7842,7 +7852,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>69.5095948827292</v>
@@ -7901,7 +7911,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>77.0788912579957</v>
@@ -7960,7 +7970,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>87.6332622601279</v>
@@ -8019,7 +8029,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>95.8422174840085</v>
@@ -8078,7 +8088,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>90.7249466950959</v>
@@ -8137,7 +8147,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>99.4669509594883</v>
@@ -8196,7 +8206,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>98.0810234541578</v>
@@ -8255,7 +8265,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>100.426439232409</v>
@@ -8314,7 +8324,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>99.680170575693</v>
@@ -8373,7 +8383,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>121.961620469083</v>
@@ -8432,7 +8442,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>150.106609808102</v>
@@ -8491,7 +8501,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>99.1471215351812</v>
@@ -8550,7 +8560,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>115.778251599147</v>
@@ -8609,7 +8619,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>118.763326226013</v>
@@ -8668,7 +8678,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>116.311300639659</v>
@@ -8727,7 +8737,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>123.347547974414</v>
@@ -8786,7 +8796,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>116.311300639659</v>
@@ -8845,7 +8855,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>116.098081023454</v>
@@ -8904,7 +8914,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>110.874200426439</v>
@@ -8963,7 +8973,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>125.266524520256</v>
@@ -9022,7 +9032,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>128.678038379531</v>
@@ -9081,7 +9091,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>122.601279317697</v>
@@ -9140,7 +9150,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>113.006396588486</v>
@@ -9199,7 +9209,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>102.985074626866</v>
@@ -9258,7 +9268,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>79.1044776119403</v>
@@ -9317,7 +9327,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>102.878464818763</v>
@@ -9376,7 +9386,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>104.371002132196</v>
@@ -9435,7 +9445,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>102.452025586354</v>
@@ -9494,7 +9504,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>103.19829424307</v>
@@ -9553,7 +9563,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>103.304904051173</v>
@@ -9612,7 +9622,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>109.488272921109</v>
@@ -9671,7 +9681,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>106.289978678038</v>
@@ -9730,7 +9740,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>105.650319829424</v>
@@ -9789,7 +9799,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>106.503198294243</v>
@@ -9848,7 +9858,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>106.503198294243</v>
@@ -9907,7 +9917,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>103.62473347548</v>
@@ -9966,7 +9976,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>102.771855010661</v>
@@ -10025,7 +10035,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>102.771855010661</v>
@@ -10084,7 +10094,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>102.238805970149</v>
@@ -10143,7 +10153,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>101.172707889126</v>
@@ -10202,7 +10212,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>105.863539445629</v>
@@ -10261,7 +10271,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>103.518123667377</v>
@@ -10320,7 +10330,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>92.0042643923241</v>
@@ -10379,7 +10389,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>76.226012793177</v>
@@ -10438,7 +10448,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>79.4243070362473</v>
@@ -10497,7 +10507,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>93.1769722814499</v>
@@ -10556,7 +10566,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>98.8272921108742</v>
@@ -10615,7 +10625,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>98.8272921108742</v>
@@ -10674,7 +10684,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>83.2622601279318</v>
@@ -10733,7 +10743,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>89.8720682302772</v>
@@ -10792,7 +10802,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>95.4157782515991</v>
@@ -10851,7 +10861,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>101.066098081023</v>
@@ -10910,7 +10920,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>109.701492537313</v>
@@ -10969,7 +10979,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>104.797441364606</v>
@@ -11028,7 +11038,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>125.479744136461</v>
@@ -11087,7 +11097,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>133.795309168443</v>
@@ -11146,7 +11156,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>132.196162046908</v>
@@ -11205,7 +11215,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>117.803837953092</v>
@@ -11264,7 +11274,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>110.554371002132</v>
@@ -11323,7 +11333,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>103.518123667377</v>
@@ -11382,7 +11392,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>106.076759061834</v>
@@ -11441,7 +11451,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>104.477611940299</v>
@@ -11500,7 +11510,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>103.837953091684</v>
@@ -11559,7 +11569,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>102.132196162047</v>
@@ -11618,7 +11628,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>105.117270788913</v>
@@ -11677,7 +11687,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>102.238805970149</v>
@@ -11736,7 +11746,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>101.066098081023</v>
@@ -11795,7 +11805,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>101.492537313433</v>
@@ -11854,7 +11864,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>100.639658848614</v>
@@ -11913,7 +11923,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>105.970149253731</v>
@@ -11972,7 +11982,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>103.19829424307</v>
@@ -12031,7 +12041,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>105.330490405117</v>
@@ -12090,7 +12100,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2"/>
       <c r="C175" s="3" t="n">
@@ -12123,7 +12133,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2"/>
       <c r="C176" s="3" t="n">
@@ -12156,7 +12166,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2"/>
       <c r="C177" s="3" t="n">
@@ -12189,7 +12199,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2"/>
       <c r="C178" s="3" t="n">
@@ -12222,7 +12232,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2"/>
       <c r="C179" s="3" t="n">
@@ -12255,7 +12265,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2"/>
       <c r="C180" s="3" t="n">
@@ -12288,7 +12298,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2"/>
       <c r="C181" s="3" t="n">
@@ -12321,7 +12331,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2"/>
       <c r="C182" s="3" t="n">
@@ -12354,7 +12364,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2"/>
       <c r="C183" s="3" t="n">
@@ -12387,7 +12397,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2"/>
       <c r="C184" s="3" t="n">
@@ -12420,7 +12430,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2"/>
       <c r="C185" s="3" t="n">
@@ -12453,7 +12463,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2"/>
       <c r="C186" s="3" t="n">
@@ -12486,7 +12496,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2"/>
       <c r="C187" s="3"/>
@@ -12509,7 +12519,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2"/>
       <c r="C188" s="3"/>
@@ -12532,7 +12542,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2"/>
       <c r="C189" s="3"/>
@@ -12555,7 +12565,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2"/>
       <c r="C190" s="3"/>
@@ -12578,7 +12588,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2"/>
       <c r="C191" s="3"/>
@@ -12601,7 +12611,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2"/>
       <c r="C192" s="3"/>
@@ -12624,7 +12634,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2"/>
       <c r="C193" s="3"/>
@@ -12647,7 +12657,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2"/>
       <c r="C194" s="3"/>
@@ -12670,7 +12680,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2"/>
       <c r="C195" s="3"/>
@@ -12693,7 +12703,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2"/>
       <c r="C196" s="3"/>
@@ -12716,7 +12726,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2"/>
       <c r="C197" s="3"/>
@@ -12739,7 +12749,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2"/>
       <c r="C198" s="3"/>
@@ -12762,7 +12772,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2"/>
       <c r="C199" s="3"/>
@@ -12785,7 +12795,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2"/>
       <c r="C200" s="3"/>
@@ -12808,7 +12818,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2"/>
       <c r="C201" s="3"/>
@@ -12831,7 +12841,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2"/>
       <c r="C202" s="3"/>
@@ -12854,7 +12864,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2"/>
       <c r="C203" s="3"/>
@@ -12877,7 +12887,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2"/>
       <c r="C204" s="3"/>
@@ -12900,7 +12910,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2"/>
       <c r="C205" s="3"/>
@@ -12923,7 +12933,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2"/>
       <c r="C206" s="3"/>
@@ -12946,7 +12956,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2"/>
       <c r="C207" s="3"/>
@@ -12969,7 +12979,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2"/>
       <c r="C208" s="3"/>
@@ -12992,7 +13002,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2"/>
       <c r="C209" s="3"/>
@@ -13015,7 +13025,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2"/>
       <c r="C210" s="3"/>
@@ -13038,7 +13048,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2"/>
       <c r="C211" s="3"/>
@@ -13061,7 +13071,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2"/>
       <c r="C212" s="3"/>
@@ -13084,7 +13094,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2"/>
       <c r="C213" s="3"/>
@@ -13107,7 +13117,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2"/>
       <c r="C214" s="3"/>
@@ -13130,7 +13140,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2"/>
       <c r="C215" s="3"/>
@@ -13153,7 +13163,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2"/>
       <c r="C216" s="3"/>
@@ -13176,7 +13186,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2"/>
       <c r="C217" s="3"/>
@@ -13199,7 +13209,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2"/>
       <c r="C218" s="3"/>
@@ -13222,7 +13232,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2"/>
       <c r="C219" s="3"/>
@@ -13245,7 +13255,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2"/>
       <c r="C220" s="3"/>
@@ -13268,7 +13278,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2"/>
       <c r="C221" s="3"/>
@@ -13291,7 +13301,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2"/>
       <c r="C222" s="3"/>
@@ -13314,7 +13324,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2"/>
       <c r="C223" s="3"/>
@@ -13337,7 +13347,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2"/>
       <c r="C224" s="3"/>
@@ -13360,7 +13370,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2"/>
       <c r="C225" s="3"/>
@@ -13383,7 +13393,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2"/>
       <c r="C226" s="3"/>
@@ -13406,7 +13416,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2"/>
       <c r="C227" s="3"/>
@@ -13429,7 +13439,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2"/>
       <c r="C228" s="3"/>
@@ -13452,7 +13462,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2"/>
       <c r="C229" s="3"/>
@@ -13486,97 +13496,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -13600,7 +13610,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -13610,13 +13620,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>-0.0715650415336092</v>
@@ -13624,7 +13634,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>-0.058070371125012</v>
@@ -13632,7 +13642,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>-0.0666813417969528</v>
@@ -13640,7 +13650,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>-0.0990609223244074</v>
@@ -13648,7 +13658,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>-0.072988701800681</v>
@@ -13656,7 +13666,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.0638103344984167</v>
@@ -13664,7 +13674,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.247340427195767</v>
@@ -13672,7 +13682,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.397247477636655</v>
@@ -13680,7 +13690,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.491932458988993</v>
@@ -13688,7 +13698,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.536611195215531</v>
@@ -13696,7 +13706,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.478656019152781</v>
@@ -13704,7 +13714,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.337169782248179</v>
@@ -13712,7 +13722,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.245998745707208</v>
@@ -13720,7 +13730,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.22185686739852</v>
@@ -13728,7 +13738,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.157023384524968</v>
@@ -13736,7 +13746,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.0626413325924589</v>
@@ -13744,7 +13754,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.0472357908675468</v>
@@ -13752,7 +13762,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.183615750764389</v>
@@ -13760,7 +13770,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.291734174281005</v>

</xml_diff>